<commit_message>
feat: add % to tables instead of Percent and change number format to 0dp
</commit_message>
<xml_diff>
--- a/data/common_project_data/indicators-master.xlsx
+++ b/data/common_project_data/indicators-master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve.crawshaw\projects\weca_regional_indicators\data\common_project_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF194CCE-6CAF-4DBB-9727-AB0C6D11AE12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED97C362-6935-463D-B7F6-0A254EF57198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2286,9 +2286,6 @@
     <t>All indicator metadata — units, geography level, data source, definition, polarity — lives exclusively in dim_indicator and is resolved via FK join.</t>
   </si>
   <si>
-    <t>Percent</t>
-  </si>
-  <si>
     <t>ONS Labour Force Survey</t>
   </si>
   <si>
@@ -2680,6 +2677,9 @@
   </si>
   <si>
     <t>include</t>
+  </si>
+  <si>
+    <t>%</t>
   </si>
 </sst>
 </file>
@@ -9748,16 +9748,16 @@
         <v>37</v>
       </c>
       <c r="AM1" s="26" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="AN1" s="3" t="s">
         <v>38</v>
       </c>
       <c r="AO1" s="3" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="AP1" s="3" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="AQ1" s="2"/>
     </row>
@@ -9877,16 +9877,16 @@
         <v>76</v>
       </c>
       <c r="AM2" s="27" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="AN2" s="12" t="s">
         <v>77</v>
       </c>
       <c r="AO2" s="12" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="AP2" s="12" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="AQ2" s="2"/>
     </row>
@@ -9910,13 +9910,13 @@
         <v>83</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="H3" s="1">
         <v>1</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>84</v>
@@ -9926,13 +9926,13 @@
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="N3" s="1" t="s">
         <v>731</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="O3" s="11" t="s">
         <v>732</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>733</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>117</v>
@@ -9944,7 +9944,7 @@
         <v>183</v>
       </c>
       <c r="S3" s="1" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="T3" s="23">
         <v>46133</v>
@@ -9953,10 +9953,10 @@
         <v>4</v>
       </c>
       <c r="W3" s="1" t="s">
+        <v>735</v>
+      </c>
+      <c r="Y3" s="1" t="s">
         <v>736</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>737</v>
       </c>
       <c r="Z3" s="1" t="s">
         <v>88</v>
@@ -9965,7 +9965,7 @@
         <v>173</v>
       </c>
       <c r="AB3" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="AC3" s="1" t="s">
         <v>89</v>
@@ -9978,13 +9978,13 @@
         <v>91</v>
       </c>
       <c r="AL3" s="1" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="AM3" s="5">
         <v>3</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP3" s="1" t="b">
         <v>1</v>
@@ -10010,13 +10010,13 @@
         <v>94</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>95</v>
@@ -10026,13 +10026,13 @@
         <v>86</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>741</v>
+      </c>
+      <c r="O4" s="11" t="s">
+        <v>740</v>
+      </c>
+      <c r="P4" s="1" t="s">
         <v>742</v>
-      </c>
-      <c r="O4" s="11" t="s">
-        <v>741</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>743</v>
       </c>
       <c r="Q4" s="1" t="s">
         <v>457</v>
@@ -10053,13 +10053,13 @@
         <v>98</v>
       </c>
       <c r="W4" s="1" t="s">
+        <v>743</v>
+      </c>
+      <c r="X4" s="1" t="s">
+        <v>750</v>
+      </c>
+      <c r="Y4" s="1" t="s">
         <v>744</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>751</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>745</v>
       </c>
       <c r="Z4" s="1" t="s">
         <v>88</v>
@@ -10068,7 +10068,7 @@
         <v>509</v>
       </c>
       <c r="AB4" s="1" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="AC4" s="1" t="s">
         <v>89</v>
@@ -10084,7 +10084,7 @@
         <v>4</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP4" s="1" t="b">
         <v>1</v>
@@ -10110,16 +10110,16 @@
         <v>103</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="H5" s="1">
         <v>1</v>
       </c>
       <c r="I5" s="1" t="s">
+        <v>746</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>747</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>748</v>
       </c>
       <c r="L5" s="5">
         <v>2020</v>
@@ -10128,10 +10128,10 @@
         <v>104</v>
       </c>
       <c r="N5" s="1" t="s">
+        <v>748</v>
+      </c>
+      <c r="O5" s="11" t="s">
         <v>749</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>750</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>105</v>
@@ -10146,19 +10146,19 @@
         <v>2023</v>
       </c>
       <c r="T5" s="24" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="U5" s="1">
         <v>16</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="X5" s="1" t="s">
+        <v>751</v>
+      </c>
+      <c r="Y5" s="1" t="s">
         <v>752</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>753</v>
       </c>
       <c r="Z5" s="1" t="s">
         <v>88</v>
@@ -10167,7 +10167,7 @@
         <v>509</v>
       </c>
       <c r="AB5" s="1" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="AC5" s="1" t="s">
         <v>89</v>
@@ -10183,7 +10183,7 @@
         <v>1</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="AP5" s="1" t="b">
         <v>1</v>
@@ -10209,7 +10209,7 @@
         <v>110</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="H6" s="1">
         <v>1</v>
@@ -10218,20 +10218,20 @@
         <v>111</v>
       </c>
       <c r="J6" s="1" t="s">
+        <v>758</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>759</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>760</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="1" t="s">
+        <v>760</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>761</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="11" t="s">
         <v>762</v>
-      </c>
-      <c r="O6" s="11" t="s">
-        <v>763</v>
       </c>
       <c r="P6" s="1" t="s">
         <v>105</v>
@@ -10252,10 +10252,10 @@
         <v>18</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="Y6" s="1" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="Z6" s="1" t="s">
         <v>88</v>
@@ -10264,7 +10264,7 @@
         <v>173</v>
       </c>
       <c r="AB6" s="1" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="AC6" s="1" t="s">
         <v>89</v>
@@ -10277,13 +10277,13 @@
         <v>113</v>
       </c>
       <c r="AL6" s="1" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="AM6" s="5">
         <v>2</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="AP6" s="1" t="b">
         <v>1</v>
@@ -10306,10 +10306,10 @@
         <v>115</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>768</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>769</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>770</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
@@ -10318,23 +10318,23 @@
         <v>116</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="L7" s="5"/>
       <c r="M7" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>771</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="O7" s="11" t="s">
         <v>772</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>773</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>117</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="R7" s="1" t="s">
         <v>87</v>
@@ -10349,10 +10349,10 @@
         <v>1</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="Z7" s="1" t="s">
         <v>88</v>
@@ -10361,7 +10361,7 @@
         <v>437</v>
       </c>
       <c r="AB7" s="1" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="AC7" s="1" t="s">
         <v>89</v>
@@ -10374,13 +10374,13 @@
         <v>91</v>
       </c>
       <c r="AL7" s="1" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="AM7" s="5">
         <v>5</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="AP7" s="1" t="b">
         <v>1</v>
@@ -10406,13 +10406,13 @@
         <v>121</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="H8" s="1">
         <v>1</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>122</v>
@@ -10428,13 +10428,13 @@
         <v>124</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>38</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="R8" s="1" t="s">
         <v>125</v>
@@ -10449,10 +10449,10 @@
         <v>18</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="Z8" s="1" t="s">
         <v>88</v>
@@ -10461,7 +10461,7 @@
         <v>509</v>
       </c>
       <c r="AB8" s="1" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="AC8" s="1" t="s">
         <v>89</v>
@@ -10477,7 +10477,7 @@
         <v>12</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP8" s="1" t="b">
         <v>0</v>
@@ -10500,26 +10500,26 @@
         <v>130</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="H9" s="1">
         <v>1</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>131</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="1" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>132</v>
@@ -10534,7 +10534,7 @@
         <v>5</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="Z9" s="1" t="s">
         <v>88</v>
@@ -10550,13 +10550,13 @@
         <v>91</v>
       </c>
       <c r="AL9" s="1" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="AM9" s="5">
         <v>6</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP9" s="1" t="b">
         <v>1</v>
@@ -10582,32 +10582,32 @@
         <v>136</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="H10" s="1">
         <v>1</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="1" t="s">
         <v>137</v>
       </c>
       <c r="N10" s="1" t="s">
+        <v>779</v>
+      </c>
+      <c r="O10" s="11" t="s">
         <v>780</v>
-      </c>
-      <c r="O10" s="11" t="s">
-        <v>781</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>117</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="R10" s="1" t="s">
         <v>506</v>
@@ -10616,13 +10616,13 @@
         <v>46054</v>
       </c>
       <c r="T10" s="1" t="s">
+        <v>783</v>
+      </c>
+      <c r="V10" s="1" t="s">
         <v>784</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="W10" s="1" t="s">
         <v>785</v>
-      </c>
-      <c r="W10" s="1" t="s">
-        <v>786</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>138</v>
@@ -10644,7 +10644,7 @@
         <v>7</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP10" s="1" t="b">
         <v>0</v>
@@ -10722,7 +10722,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>152</v>
@@ -10760,7 +10760,7 @@
         <v>9</v>
       </c>
       <c r="AO12" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP12" s="1" t="b">
         <v>1</v>
@@ -10789,7 +10789,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>160</v>
@@ -10833,7 +10833,7 @@
         <v>11</v>
       </c>
       <c r="AO13" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP13" s="1" t="b">
         <v>1</v>
@@ -10859,32 +10859,32 @@
         <v>170</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="H14" s="1">
         <v>1</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J14" s="1" t="s">
+        <v>828</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>829</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>830</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="1" t="s">
         <v>171</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="Q14" s="1" t="s">
         <v>457</v>
@@ -10893,22 +10893,22 @@
         <v>125</v>
       </c>
       <c r="S14" s="1" t="s">
+        <v>794</v>
+      </c>
+      <c r="T14" s="1" t="s">
         <v>795</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>796</v>
       </c>
       <c r="U14" s="1">
         <v>8</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="X14" s="1" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>172</v>
@@ -10920,7 +10920,7 @@
         <v>509</v>
       </c>
       <c r="AB14" s="1" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="AC14" s="1" t="s">
         <v>89</v>
@@ -10945,7 +10945,7 @@
         <v>177</v>
       </c>
       <c r="AO14" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP14" s="1" t="b">
         <v>1</v>
@@ -10971,26 +10971,26 @@
         <v>181</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="H15" s="1">
         <v>1</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>182</v>
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="1" t="s">
+        <v>835</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="O15" s="11" t="s">
         <v>836</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>838</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>837</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>132</v>
@@ -11002,10 +11002,10 @@
         <v>96</v>
       </c>
       <c r="S15" s="1" t="s">
+        <v>838</v>
+      </c>
+      <c r="T15" s="1" t="s">
         <v>839</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>840</v>
       </c>
       <c r="U15" s="1">
         <v>9</v>
@@ -11014,7 +11014,7 @@
         <v>184</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="Y15" s="1" t="s">
         <v>185</v>
@@ -11045,7 +11045,7 @@
         <v>188</v>
       </c>
       <c r="AO15" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP15" s="1" t="b">
         <v>1</v>
@@ -11068,22 +11068,22 @@
         <v>190</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="H16" s="1">
         <v>1</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>191</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="1" t="s">
@@ -11102,7 +11102,7 @@
         <v>194</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="Y16" s="1" t="s">
         <v>195</v>
@@ -11130,7 +11130,7 @@
         <v>188</v>
       </c>
       <c r="AO16" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP16" s="1" t="b">
         <v>1</v>
@@ -11153,16 +11153,16 @@
         <v>199</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="H17" s="1">
         <v>1</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>200</v>
@@ -11215,7 +11215,7 @@
         <v>175</v>
       </c>
       <c r="AO17" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP17" s="1" t="b">
         <v>1</v>
@@ -11241,13 +11241,13 @@
         <v>207</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="H18" s="1">
         <v>1</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>208</v>
@@ -11282,7 +11282,7 @@
         <v>6</v>
       </c>
       <c r="AO18" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP18" s="1" t="b">
         <v>1</v>
@@ -11308,19 +11308,19 @@
         <v>214</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="H19" s="1">
         <v>1</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>831</v>
+        <v>830</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="L19" s="5"/>
       <c r="M19" s="1" t="s">
@@ -11361,7 +11361,7 @@
         <v>5</v>
       </c>
       <c r="AO19" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP19" s="1" t="b">
         <v>1</v>
@@ -11384,19 +11384,19 @@
         <v>222</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>823</v>
+        <v>822</v>
       </c>
       <c r="H20" s="1">
         <v>1</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
       <c r="L20" s="5"/>
       <c r="M20" s="1" t="s">
@@ -11440,7 +11440,7 @@
         <v>175</v>
       </c>
       <c r="AO20" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="AP20" s="1" t="b">
         <v>1</v>
@@ -11463,19 +11463,19 @@
         <v>226</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
       <c r="H21" s="1">
         <v>1</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>152</v>
@@ -11513,7 +11513,7 @@
         <v>8</v>
       </c>
       <c r="AO21" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP21" s="1" t="b">
         <v>1</v>
@@ -11576,16 +11576,16 @@
         <v>237</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="H23" s="1">
         <v>1</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>238</v>
@@ -11626,7 +11626,7 @@
         <v>3</v>
       </c>
       <c r="AO23" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP23" s="1" t="b">
         <v>1</v>
@@ -11649,13 +11649,13 @@
         <v>244</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="H24" s="1">
         <v>1</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="J24" s="1" t="s">
         <v>245</v>
@@ -11693,7 +11693,7 @@
         <v>9</v>
       </c>
       <c r="AO24" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP24" s="1" t="b">
         <v>0</v>
@@ -11757,7 +11757,7 @@
         <v>175</v>
       </c>
       <c r="AO25" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP25" s="1" t="b">
         <v>0</v>
@@ -11815,7 +11815,7 @@
         <v>11</v>
       </c>
       <c r="AO26" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP26" s="1" t="b">
         <v>1</v>
@@ -11844,7 +11844,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>271</v>
@@ -11885,7 +11885,7 @@
         <v>3</v>
       </c>
       <c r="AO27" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP27" s="1" t="b">
         <v>1</v>
@@ -11908,13 +11908,13 @@
         <v>278</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="H28" s="1">
         <v>-1</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>279</v>
@@ -11961,7 +11961,7 @@
         <v>2</v>
       </c>
       <c r="AO28" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP28" s="1" t="b">
         <v>1</v>
@@ -11984,13 +11984,13 @@
         <v>287</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="H29" s="1">
         <v>-1</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="J29" s="1" t="s">
         <v>288</v>
@@ -12034,7 +12034,7 @@
         <v>4</v>
       </c>
       <c r="AO29" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP29" s="1" t="b">
         <v>0</v>
@@ -12057,13 +12057,13 @@
         <v>297</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="H30" s="1">
         <v>1</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>298</v>
@@ -12113,7 +12113,7 @@
         <v>91</v>
       </c>
       <c r="AO30" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP30" s="1" t="b">
         <v>1</v>
@@ -12186,7 +12186,7 @@
         <v>5</v>
       </c>
       <c r="AO31" s="1" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="AP31" s="1" t="b">
         <v>1</v>
@@ -12259,7 +12259,7 @@
         <v>6</v>
       </c>
       <c r="AO32" s="1" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="AP32" s="1" t="b">
         <v>1</v>
@@ -12326,7 +12326,7 @@
         <v>7</v>
       </c>
       <c r="AO33" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP33" s="1" t="b">
         <v>1</v>
@@ -12355,7 +12355,7 @@
         <v>1</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>336</v>
@@ -12393,7 +12393,7 @@
         <v>8</v>
       </c>
       <c r="AO34" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP34" s="1" t="b">
         <v>1</v>
@@ -12468,7 +12468,7 @@
         <v>1</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="L36" s="5"/>
       <c r="R36" s="1" t="s">
@@ -12500,7 +12500,7 @@
         <v>351</v>
       </c>
       <c r="AO36" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP36" s="1" t="b">
         <v>1</v>
@@ -12529,7 +12529,7 @@
         <v>-1</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>358</v>
@@ -12570,7 +12570,7 @@
         <v>1</v>
       </c>
       <c r="AO37" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP37" s="1" t="b">
         <v>1</v>
@@ -12593,13 +12593,13 @@
         <v>365</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="H38" s="1">
         <v>1</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>366</v>
@@ -12643,7 +12643,7 @@
         <v>2</v>
       </c>
       <c r="AO38" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP38" s="1" t="b">
         <v>1</v>
@@ -12672,7 +12672,7 @@
         <v>1</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>371</v>
@@ -12713,7 +12713,7 @@
         <v>8</v>
       </c>
       <c r="AO39" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP39" s="1" t="b">
         <v>1</v>
@@ -12736,13 +12736,13 @@
         <v>377</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="H40" s="1">
         <v>1</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="1" t="s">
@@ -12783,7 +12783,7 @@
         <v>9</v>
       </c>
       <c r="AO40" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="AP40" s="1" t="b">
         <v>1</v>
@@ -12812,7 +12812,7 @@
         <v>1</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J41" s="1" t="s">
         <v>385</v>
@@ -12853,7 +12853,7 @@
         <v>7</v>
       </c>
       <c r="AO41" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP41" s="1" t="b">
         <v>1</v>
@@ -12882,7 +12882,7 @@
         <v>-1</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J42" s="1" t="s">
         <v>391</v>
@@ -12920,7 +12920,7 @@
         <v>6</v>
       </c>
       <c r="AO42" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP42" s="1" t="b">
         <v>1</v>
@@ -12949,7 +12949,7 @@
         <v>-1</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>396</v>
@@ -12996,7 +12996,7 @@
         <v>3</v>
       </c>
       <c r="AO43" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP43" s="1" t="b">
         <v>1</v>
@@ -13025,7 +13025,7 @@
         <v>-1</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="L44" s="5"/>
       <c r="Y44" s="1" t="s">
@@ -13054,7 +13054,7 @@
         <v>4</v>
       </c>
       <c r="AO44" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP44" s="1" t="b">
         <v>1</v>
@@ -13077,13 +13077,13 @@
         <v>409</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="H45" s="1">
         <v>-1</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J45" s="1" t="s">
         <v>410</v>
@@ -13127,7 +13127,7 @@
         <v>5</v>
       </c>
       <c r="AO45" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP45" s="1" t="b">
         <v>1</v>
@@ -13260,7 +13260,7 @@
         <v>5</v>
       </c>
       <c r="F48" s="22" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>431</v>
@@ -13322,7 +13322,7 @@
         <v>1</v>
       </c>
       <c r="AO48" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP48" s="1" t="b">
         <v>1</v>
@@ -13345,7 +13345,7 @@
         <v>442</v>
       </c>
       <c r="F49" s="22" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>443</v>
@@ -13410,7 +13410,7 @@
         <v>10</v>
       </c>
       <c r="AO49" s="1" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AP49" s="1" t="b">
         <v>1</v>
@@ -13433,7 +13433,7 @@
         <v>452</v>
       </c>
       <c r="F50" s="22" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>453</v>
@@ -13442,7 +13442,7 @@
         <v>1</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="J50" s="1" t="s">
         <v>454</v>
@@ -13507,7 +13507,7 @@
         <v>9</v>
       </c>
       <c r="AO50" s="1" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AP50" s="1" t="b">
         <v>1</v>
@@ -13539,7 +13539,7 @@
         <v>1</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J51" s="1" t="s">
         <v>466</v>
@@ -13598,7 +13598,7 @@
         <v>8</v>
       </c>
       <c r="AO51" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP51" s="1" t="b">
         <v>1</v>
@@ -13686,7 +13686,7 @@
         <v>2</v>
       </c>
       <c r="AO52" s="1" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AP52" s="1" t="b">
         <v>1</v>
@@ -13709,7 +13709,7 @@
         <v>488</v>
       </c>
       <c r="F53" s="22" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>489</v>
@@ -13767,7 +13767,7 @@
         <v>3</v>
       </c>
       <c r="AO53" s="1" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="AP53" s="1" t="b">
         <v>1</v>
@@ -13846,7 +13846,7 @@
         <v>7</v>
       </c>
       <c r="AO54" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP54" s="1" t="b">
         <v>1</v>
@@ -13973,7 +13973,7 @@
         <v>523</v>
       </c>
       <c r="F57" s="22" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>524</v>
@@ -13982,7 +13982,7 @@
         <v>1</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J57" s="1" t="s">
         <v>525</v>
@@ -14038,7 +14038,7 @@
         <v>4</v>
       </c>
       <c r="AO57" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP57" s="1" t="b">
         <v>1</v>
@@ -14061,13 +14061,13 @@
         <v>539</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="H58" s="1">
         <v>-1</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>540</v>
@@ -14114,7 +14114,7 @@
         <v>91</v>
       </c>
       <c r="AO58" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP58" s="1" t="b">
         <v>1</v>
@@ -14143,7 +14143,7 @@
         <v>1</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J59" s="1" t="s">
         <v>548</v>
@@ -14193,7 +14193,7 @@
         <v>91</v>
       </c>
       <c r="AO59" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP59" s="1" t="b">
         <v>1</v>
@@ -14216,7 +14216,7 @@
         <v>553</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>554</v>
@@ -14225,7 +14225,7 @@
         <v>1</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J60" s="1" t="s">
         <v>555</v>
@@ -14272,7 +14272,7 @@
         <v>8</v>
       </c>
       <c r="AO60" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP60" s="1" t="b">
         <v>1</v>
@@ -14301,7 +14301,7 @@
         <v>-1</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J61" s="1" t="s">
         <v>561</v>
@@ -14345,7 +14345,7 @@
         <v>6</v>
       </c>
       <c r="AO61" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP61" s="1" t="b">
         <v>1</v>
@@ -14374,7 +14374,7 @@
         <v>1</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J62" s="1" t="s">
         <v>568</v>
@@ -14415,7 +14415,7 @@
         <v>2</v>
       </c>
       <c r="AO62" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP62" s="1" t="b">
         <v>1</v>
@@ -14444,7 +14444,7 @@
         <v>1</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J63" s="1" t="s">
         <v>576</v>
@@ -14485,7 +14485,7 @@
         <v>3</v>
       </c>
       <c r="AO63" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP63" s="1" t="b">
         <v>1</v>
@@ -14647,7 +14647,7 @@
         <v>10</v>
       </c>
       <c r="AO66" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP66" s="1" t="b">
         <v>1</v>
@@ -14717,7 +14717,7 @@
         <v>11</v>
       </c>
       <c r="AO67" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="AP67" s="1" t="b">
         <v>1</v>
@@ -14740,13 +14740,13 @@
         <v>605</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="H68" s="1">
         <v>1</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J68" s="1" t="s">
         <v>606</v>
@@ -14793,7 +14793,7 @@
         <v>4</v>
       </c>
       <c r="AO68" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP68" s="1" t="b">
         <v>1</v>
@@ -14822,7 +14822,7 @@
         <v>-1</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>730</v>
+        <v>860</v>
       </c>
       <c r="J69" s="1" t="s">
         <v>611</v>
@@ -14866,7 +14866,7 @@
         <v>7</v>
       </c>
       <c r="AO69" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP69" s="1" t="b">
         <v>1</v>
@@ -15153,33 +15153,33 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>848</v>
+      </c>
+      <c r="B10" t="s">
         <v>849</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>850</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>851</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>852</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>853</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>854</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>855</v>
-      </c>
-      <c r="H10" t="s">
-        <v>856</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="B11" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
fix: gdp growth updated
</commit_message>
<xml_diff>
--- a/data/common_project_data/indicators-master.xlsx
+++ b/data/common_project_data/indicators-master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve.crawshaw\projects\weca_regional_indicators\data\common_project_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9540A400-0674-4C41-BF7C-746DDBFEB218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5BD7C984-3BAE-465E-B390-E09C55F62ADA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1693" uniqueCount="860">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1693" uniqueCount="859">
   <si>
     <t>Unique ID</t>
   </si>
@@ -2317,9 +2317,6 @@
   </si>
   <si>
     <t>The data for priority sectors goes down to very low SIC (industry) levels where the data are less reliable.</t>
-  </si>
-  <si>
-    <t>Index</t>
   </si>
   <si>
     <t>GDP level indexed to 2020</t>
@@ -9745,16 +9742,16 @@
         <v>37</v>
       </c>
       <c r="AM1" s="26" t="s">
-        <v>808</v>
+        <v>807</v>
       </c>
       <c r="AN1" s="3" t="s">
         <v>38</v>
       </c>
       <c r="AO1" s="3" t="s">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="AP1" s="3" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="AQ1" s="2"/>
     </row>
@@ -9874,16 +9871,16 @@
         <v>76</v>
       </c>
       <c r="AM2" s="27" t="s">
-        <v>809</v>
+        <v>808</v>
       </c>
       <c r="AN2" s="12" t="s">
         <v>77</v>
       </c>
       <c r="AO2" s="12" t="s">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="AP2" s="12" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="AQ2" s="2"/>
     </row>
@@ -9907,13 +9904,13 @@
         <v>83</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="H3" s="1">
         <v>1</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>84</v>
@@ -9981,7 +9978,7 @@
         <v>3</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP3" s="1" t="b">
         <v>1</v>
@@ -10007,7 +10004,7 @@
         <v>94</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="H4" s="1">
         <v>1</v>
@@ -10053,7 +10050,7 @@
         <v>738</v>
       </c>
       <c r="X4" s="1" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>739</v>
@@ -10081,7 +10078,7 @@
         <v>4</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP4" s="1" t="b">
         <v>1</v>
@@ -10107,16 +10104,16 @@
         <v>103</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="H5" s="1">
         <v>1</v>
       </c>
       <c r="I5" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>741</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>742</v>
       </c>
       <c r="L5" s="5">
         <v>2020</v>
@@ -10125,10 +10122,10 @@
         <v>104</v>
       </c>
       <c r="N5" s="1" t="s">
+        <v>742</v>
+      </c>
+      <c r="O5" s="11" t="s">
         <v>743</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>744</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>105</v>
@@ -10143,7 +10140,7 @@
         <v>2023</v>
       </c>
       <c r="T5" s="24" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="U5" s="1">
         <v>16</v>
@@ -10152,10 +10149,10 @@
         <v>738</v>
       </c>
       <c r="X5" s="1" t="s">
+        <v>745</v>
+      </c>
+      <c r="Y5" s="1" t="s">
         <v>746</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>747</v>
       </c>
       <c r="Z5" s="1" t="s">
         <v>88</v>
@@ -10164,7 +10161,7 @@
         <v>504</v>
       </c>
       <c r="AB5" s="1" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="AC5" s="1" t="s">
         <v>89</v>
@@ -10180,7 +10177,7 @@
         <v>1</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="AP5" s="1" t="b">
         <v>1</v>
@@ -10188,7 +10185,7 @@
     </row>
     <row r="6" spans="1:43" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>79</v>
@@ -10203,10 +10200,10 @@
         <v>108</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="H6" s="1">
         <v>1</v>
@@ -10215,20 +10212,20 @@
         <v>112</v>
       </c>
       <c r="J6" s="1" t="s">
+        <v>752</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>753</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>754</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="1" t="s">
+        <v>754</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>755</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="11" t="s">
         <v>756</v>
-      </c>
-      <c r="O6" s="11" t="s">
-        <v>757</v>
       </c>
       <c r="P6" s="1" t="s">
         <v>105</v>
@@ -10252,7 +10249,7 @@
         <v>738</v>
       </c>
       <c r="Y6" s="1" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="Z6" s="1" t="s">
         <v>88</v>
@@ -10261,7 +10258,7 @@
         <v>169</v>
       </c>
       <c r="AB6" s="1" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="AC6" s="1" t="s">
         <v>89</v>
@@ -10274,13 +10271,13 @@
         <v>110</v>
       </c>
       <c r="AL6" s="1" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="AM6" s="5">
         <v>2</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="AP6" s="1" t="b">
         <v>1</v>
@@ -10288,7 +10285,7 @@
     </row>
     <row r="7" spans="1:43" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>79</v>
@@ -10303,10 +10300,10 @@
         <v>111</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>762</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>763</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>764</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
@@ -10315,23 +10312,23 @@
         <v>112</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="L7" s="5"/>
       <c r="M7" s="1" t="s">
+        <v>764</v>
+      </c>
+      <c r="N7" s="1" t="s">
         <v>765</v>
       </c>
-      <c r="N7" s="1" t="s">
+      <c r="O7" s="11" t="s">
         <v>766</v>
-      </c>
-      <c r="O7" s="11" t="s">
-        <v>767</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>113</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="R7" s="1" t="s">
         <v>87</v>
@@ -10349,7 +10346,7 @@
         <v>738</v>
       </c>
       <c r="Y7" s="1" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="Z7" s="1" t="s">
         <v>88</v>
@@ -10358,7 +10355,7 @@
         <v>432</v>
       </c>
       <c r="AB7" s="1" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="AC7" s="1" t="s">
         <v>89</v>
@@ -10371,13 +10368,13 @@
         <v>91</v>
       </c>
       <c r="AL7" s="1" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="AM7" s="5">
         <v>5</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="AP7" s="1" t="b">
         <v>1</v>
@@ -10403,13 +10400,13 @@
         <v>117</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="H8" s="1">
         <v>1</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>118</v>
@@ -10425,13 +10422,13 @@
         <v>120</v>
       </c>
       <c r="O8" s="11" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="P8" s="1" t="s">
         <v>38</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="R8" s="1" t="s">
         <v>121</v>
@@ -10449,7 +10446,7 @@
         <v>738</v>
       </c>
       <c r="Y8" s="1" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="Z8" s="1" t="s">
         <v>88</v>
@@ -10458,7 +10455,7 @@
         <v>504</v>
       </c>
       <c r="AB8" s="1" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="AC8" s="1" t="s">
         <v>89</v>
@@ -10474,7 +10471,7 @@
         <v>12</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP8" s="1" t="b">
         <v>0</v>
@@ -10497,26 +10494,26 @@
         <v>126</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="H9" s="1">
         <v>1</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>127</v>
       </c>
       <c r="L9" s="5"/>
       <c r="M9" s="1" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="P9" s="1" t="s">
         <v>128</v>
@@ -10531,7 +10528,7 @@
         <v>5</v>
       </c>
       <c r="Y9" s="1" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="Z9" s="1" t="s">
         <v>88</v>
@@ -10547,13 +10544,13 @@
         <v>91</v>
       </c>
       <c r="AL9" s="1" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="AM9" s="5">
         <v>6</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP9" s="1" t="b">
         <v>1</v>
@@ -10579,7 +10576,7 @@
         <v>132</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="H10" s="1">
         <v>1</v>
@@ -10588,17 +10585,17 @@
         <v>734</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="L10" s="5"/>
       <c r="M10" s="1" t="s">
         <v>133</v>
       </c>
       <c r="N10" s="1" t="s">
+        <v>773</v>
+      </c>
+      <c r="O10" s="11" t="s">
         <v>774</v>
-      </c>
-      <c r="O10" s="11" t="s">
-        <v>775</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>113</v>
@@ -10613,13 +10610,13 @@
         <v>46054</v>
       </c>
       <c r="T10" s="1" t="s">
+        <v>777</v>
+      </c>
+      <c r="V10" s="1" t="s">
         <v>778</v>
       </c>
-      <c r="V10" s="1" t="s">
+      <c r="W10" s="1" t="s">
         <v>779</v>
-      </c>
-      <c r="W10" s="1" t="s">
-        <v>780</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>134</v>
@@ -10641,7 +10638,7 @@
         <v>7</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP10" s="1" t="b">
         <v>0</v>
@@ -10719,7 +10716,7 @@
         <v>1</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>148</v>
@@ -10757,7 +10754,7 @@
         <v>9</v>
       </c>
       <c r="AO12" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP12" s="1" t="b">
         <v>1</v>
@@ -10786,7 +10783,7 @@
         <v>1</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>156</v>
@@ -10830,7 +10827,7 @@
         <v>11</v>
       </c>
       <c r="AO13" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP13" s="1" t="b">
         <v>1</v>
@@ -10856,29 +10853,29 @@
         <v>166</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="H14" s="1">
         <v>1</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J14" s="1" t="s">
+        <v>822</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>823</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>824</v>
       </c>
       <c r="L14" s="5"/>
       <c r="M14" s="1" t="s">
         <v>167</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="P14" s="1" t="s">
         <v>737</v>
@@ -10890,22 +10887,22 @@
         <v>121</v>
       </c>
       <c r="S14" s="1" t="s">
+        <v>788</v>
+      </c>
+      <c r="T14" s="1" t="s">
         <v>789</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>790</v>
       </c>
       <c r="U14" s="1">
         <v>8</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>793</v>
+        <v>792</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="X14" s="1" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>168</v>
@@ -10917,7 +10914,7 @@
         <v>504</v>
       </c>
       <c r="AB14" s="1" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="AC14" s="1" t="s">
         <v>89</v>
@@ -10942,7 +10939,7 @@
         <v>173</v>
       </c>
       <c r="AO14" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP14" s="1" t="b">
         <v>1</v>
@@ -10968,26 +10965,26 @@
         <v>177</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>813</v>
+        <v>812</v>
       </c>
       <c r="H15" s="1">
         <v>1</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>178</v>
       </c>
       <c r="L15" s="5"/>
       <c r="M15" s="1" t="s">
+        <v>829</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>831</v>
+      </c>
+      <c r="O15" s="11" t="s">
         <v>830</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>832</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>831</v>
       </c>
       <c r="P15" s="1" t="s">
         <v>128</v>
@@ -10999,10 +10996,10 @@
         <v>96</v>
       </c>
       <c r="S15" s="1" t="s">
+        <v>832</v>
+      </c>
+      <c r="T15" s="1" t="s">
         <v>833</v>
-      </c>
-      <c r="T15" s="1" t="s">
-        <v>834</v>
       </c>
       <c r="U15" s="1">
         <v>9</v>
@@ -11011,7 +11008,7 @@
         <v>180</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="Y15" s="1" t="s">
         <v>181</v>
@@ -11042,7 +11039,7 @@
         <v>184</v>
       </c>
       <c r="AO15" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP15" s="1" t="b">
         <v>1</v>
@@ -11065,22 +11062,22 @@
         <v>186</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>814</v>
+        <v>813</v>
       </c>
       <c r="H16" s="1">
         <v>1</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J16" s="1" t="s">
         <v>187</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="L16" s="5"/>
       <c r="M16" s="1" t="s">
@@ -11099,7 +11096,7 @@
         <v>190</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="Y16" s="1" t="s">
         <v>191</v>
@@ -11127,7 +11124,7 @@
         <v>184</v>
       </c>
       <c r="AO16" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP16" s="1" t="b">
         <v>1</v>
@@ -11150,16 +11147,16 @@
         <v>195</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="H17" s="1">
         <v>1</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J17" s="1" t="s">
         <v>196</v>
@@ -11212,7 +11209,7 @@
         <v>171</v>
       </c>
       <c r="AO17" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP17" s="1" t="b">
         <v>1</v>
@@ -11238,13 +11235,13 @@
         <v>203</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="H18" s="1">
         <v>1</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>822</v>
+        <v>821</v>
       </c>
       <c r="J18" s="1" t="s">
         <v>204</v>
@@ -11279,7 +11276,7 @@
         <v>6</v>
       </c>
       <c r="AO18" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP18" s="1" t="b">
         <v>1</v>
@@ -11305,19 +11302,19 @@
         <v>210</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>821</v>
+        <v>820</v>
       </c>
       <c r="H19" s="1">
         <v>1</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>829</v>
+        <v>828</v>
       </c>
       <c r="L19" s="5"/>
       <c r="M19" s="1" t="s">
@@ -11358,7 +11355,7 @@
         <v>5</v>
       </c>
       <c r="AO19" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP19" s="1" t="b">
         <v>1</v>
@@ -11381,19 +11378,19 @@
         <v>218</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>820</v>
+        <v>819</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="H20" s="1">
         <v>1</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="L20" s="5"/>
       <c r="M20" s="1" t="s">
@@ -11437,7 +11434,7 @@
         <v>171</v>
       </c>
       <c r="AO20" s="1" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="AP20" s="1" t="b">
         <v>1</v>
@@ -11460,19 +11457,19 @@
         <v>222</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>818</v>
+        <v>817</v>
       </c>
       <c r="H21" s="1">
         <v>1</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>827</v>
+        <v>826</v>
       </c>
       <c r="K21" s="1" t="s">
         <v>148</v>
@@ -11510,7 +11507,7 @@
         <v>8</v>
       </c>
       <c r="AO21" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP21" s="1" t="b">
         <v>1</v>
@@ -11573,16 +11570,16 @@
         <v>233</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="H23" s="1">
         <v>1</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J23" s="1" t="s">
         <v>234</v>
@@ -11623,7 +11620,7 @@
         <v>3</v>
       </c>
       <c r="AO23" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP23" s="1" t="b">
         <v>1</v>
@@ -11646,7 +11643,7 @@
         <v>240</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="H24" s="1">
         <v>1</v>
@@ -11690,7 +11687,7 @@
         <v>9</v>
       </c>
       <c r="AO24" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP24" s="1" t="b">
         <v>0</v>
@@ -11754,7 +11751,7 @@
         <v>171</v>
       </c>
       <c r="AO25" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP25" s="1" t="b">
         <v>0</v>
@@ -11812,7 +11809,7 @@
         <v>11</v>
       </c>
       <c r="AO26" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP26" s="1" t="b">
         <v>1</v>
@@ -11841,7 +11838,7 @@
         <v>1</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>267</v>
@@ -11882,7 +11879,7 @@
         <v>3</v>
       </c>
       <c r="AO27" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP27" s="1" t="b">
         <v>1</v>
@@ -11905,13 +11902,13 @@
         <v>274</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="H28" s="1">
         <v>-1</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J28" s="1" t="s">
         <v>275</v>
@@ -11958,7 +11955,7 @@
         <v>2</v>
       </c>
       <c r="AO28" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP28" s="1" t="b">
         <v>1</v>
@@ -11981,7 +11978,7 @@
         <v>283</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="H29" s="1">
         <v>-1</v>
@@ -12031,7 +12028,7 @@
         <v>4</v>
       </c>
       <c r="AO29" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP29" s="1" t="b">
         <v>0</v>
@@ -12054,13 +12051,13 @@
         <v>293</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="H30" s="1">
         <v>1</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>812</v>
+        <v>811</v>
       </c>
       <c r="J30" s="1" t="s">
         <v>294</v>
@@ -12110,7 +12107,7 @@
         <v>91</v>
       </c>
       <c r="AO30" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP30" s="1" t="b">
         <v>1</v>
@@ -12183,7 +12180,7 @@
         <v>5</v>
       </c>
       <c r="AO31" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP31" s="1" t="b">
         <v>1</v>
@@ -12206,7 +12203,7 @@
         <v>313</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="H32" s="1">
         <v>1</v>
@@ -12256,7 +12253,7 @@
         <v>6</v>
       </c>
       <c r="AO32" s="1" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="AP32" s="1" t="b">
         <v>1</v>
@@ -12323,7 +12320,7 @@
         <v>7</v>
       </c>
       <c r="AO33" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP33" s="1" t="b">
         <v>1</v>
@@ -12352,7 +12349,7 @@
         <v>1</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J34" s="1" t="s">
         <v>331</v>
@@ -12390,7 +12387,7 @@
         <v>8</v>
       </c>
       <c r="AO34" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP34" s="1" t="b">
         <v>1</v>
@@ -12465,7 +12462,7 @@
         <v>1</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="L36" s="5"/>
       <c r="R36" s="1" t="s">
@@ -12497,7 +12494,7 @@
         <v>346</v>
       </c>
       <c r="AO36" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP36" s="1" t="b">
         <v>1</v>
@@ -12526,7 +12523,7 @@
         <v>-1</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J37" s="1" t="s">
         <v>353</v>
@@ -12567,7 +12564,7 @@
         <v>1</v>
       </c>
       <c r="AO37" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP37" s="1" t="b">
         <v>1</v>
@@ -12590,13 +12587,13 @@
         <v>360</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="H38" s="1">
         <v>1</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>361</v>
@@ -12640,7 +12637,7 @@
         <v>2</v>
       </c>
       <c r="AO38" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP38" s="1" t="b">
         <v>1</v>
@@ -12669,7 +12666,7 @@
         <v>1</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>366</v>
@@ -12710,7 +12707,7 @@
         <v>8</v>
       </c>
       <c r="AO39" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP39" s="1" t="b">
         <v>1</v>
@@ -12733,13 +12730,13 @@
         <v>372</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
       <c r="H40" s="1">
         <v>1</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="L40" s="5"/>
       <c r="M40" s="1" t="s">
@@ -12780,7 +12777,7 @@
         <v>9</v>
       </c>
       <c r="AO40" s="1" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="AP40" s="1" t="b">
         <v>1</v>
@@ -12809,7 +12806,7 @@
         <v>1</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J41" s="1" t="s">
         <v>380</v>
@@ -12850,7 +12847,7 @@
         <v>7</v>
       </c>
       <c r="AO41" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP41" s="1" t="b">
         <v>1</v>
@@ -12879,7 +12876,7 @@
         <v>-1</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J42" s="1" t="s">
         <v>386</v>
@@ -12917,7 +12914,7 @@
         <v>6</v>
       </c>
       <c r="AO42" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP42" s="1" t="b">
         <v>1</v>
@@ -12946,7 +12943,7 @@
         <v>-1</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>391</v>
@@ -12993,7 +12990,7 @@
         <v>3</v>
       </c>
       <c r="AO43" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP43" s="1" t="b">
         <v>1</v>
@@ -13022,7 +13019,7 @@
         <v>-1</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="L44" s="5"/>
       <c r="Y44" s="1" t="s">
@@ -13051,7 +13048,7 @@
         <v>4</v>
       </c>
       <c r="AO44" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP44" s="1" t="b">
         <v>1</v>
@@ -13074,13 +13071,13 @@
         <v>404</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="H45" s="1">
         <v>-1</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J45" s="1" t="s">
         <v>405</v>
@@ -13124,7 +13121,7 @@
         <v>5</v>
       </c>
       <c r="AO45" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP45" s="1" t="b">
         <v>1</v>
@@ -13257,7 +13254,7 @@
         <v>5</v>
       </c>
       <c r="F48" s="22" t="s">
-        <v>795</v>
+        <v>794</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>426</v>
@@ -13319,7 +13316,7 @@
         <v>1</v>
       </c>
       <c r="AO48" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP48" s="1" t="b">
         <v>1</v>
@@ -13342,7 +13339,7 @@
         <v>437</v>
       </c>
       <c r="F49" s="22" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>438</v>
@@ -13407,7 +13404,7 @@
         <v>10</v>
       </c>
       <c r="AO49" s="1" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="AP49" s="1" t="b">
         <v>1</v>
@@ -13430,7 +13427,7 @@
         <v>447</v>
       </c>
       <c r="F50" s="22" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>448</v>
@@ -13439,7 +13436,7 @@
         <v>1</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="J50" s="1" t="s">
         <v>449</v>
@@ -13504,7 +13501,7 @@
         <v>9</v>
       </c>
       <c r="AO50" s="1" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="AP50" s="1" t="b">
         <v>1</v>
@@ -13536,7 +13533,7 @@
         <v>1</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J51" s="1" t="s">
         <v>461</v>
@@ -13595,7 +13592,7 @@
         <v>8</v>
       </c>
       <c r="AO51" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP51" s="1" t="b">
         <v>1</v>
@@ -13683,7 +13680,7 @@
         <v>2</v>
       </c>
       <c r="AO52" s="1" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="AP52" s="1" t="b">
         <v>1</v>
@@ -13706,7 +13703,7 @@
         <v>483</v>
       </c>
       <c r="F53" s="22" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="G53" s="1" t="s">
         <v>484</v>
@@ -13764,7 +13761,7 @@
         <v>3</v>
       </c>
       <c r="AO53" s="1" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="AP53" s="1" t="b">
         <v>1</v>
@@ -13843,7 +13840,7 @@
         <v>7</v>
       </c>
       <c r="AO54" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP54" s="1" t="b">
         <v>1</v>
@@ -13970,7 +13967,7 @@
         <v>518</v>
       </c>
       <c r="F57" s="22" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>519</v>
@@ -13979,7 +13976,7 @@
         <v>1</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J57" s="1" t="s">
         <v>520</v>
@@ -14035,7 +14032,7 @@
         <v>4</v>
       </c>
       <c r="AO57" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP57" s="1" t="b">
         <v>1</v>
@@ -14058,13 +14055,13 @@
         <v>534</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="H58" s="1">
         <v>-1</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J58" s="1" t="s">
         <v>535</v>
@@ -14111,7 +14108,7 @@
         <v>91</v>
       </c>
       <c r="AO58" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP58" s="1" t="b">
         <v>1</v>
@@ -14140,7 +14137,7 @@
         <v>1</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J59" s="1" t="s">
         <v>543</v>
@@ -14190,7 +14187,7 @@
         <v>91</v>
       </c>
       <c r="AO59" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP59" s="1" t="b">
         <v>1</v>
@@ -14213,7 +14210,7 @@
         <v>548</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>798</v>
+        <v>797</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>549</v>
@@ -14222,7 +14219,7 @@
         <v>1</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J60" s="1" t="s">
         <v>550</v>
@@ -14269,7 +14266,7 @@
         <v>8</v>
       </c>
       <c r="AO60" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP60" s="1" t="b">
         <v>1</v>
@@ -14298,7 +14295,7 @@
         <v>-1</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J61" s="1" t="s">
         <v>556</v>
@@ -14342,7 +14339,7 @@
         <v>6</v>
       </c>
       <c r="AO61" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP61" s="1" t="b">
         <v>1</v>
@@ -14371,7 +14368,7 @@
         <v>1</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J62" s="1" t="s">
         <v>563</v>
@@ -14412,7 +14409,7 @@
         <v>2</v>
       </c>
       <c r="AO62" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP62" s="1" t="b">
         <v>1</v>
@@ -14441,7 +14438,7 @@
         <v>1</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J63" s="1" t="s">
         <v>571</v>
@@ -14482,7 +14479,7 @@
         <v>3</v>
       </c>
       <c r="AO63" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP63" s="1" t="b">
         <v>1</v>
@@ -14644,7 +14641,7 @@
         <v>10</v>
       </c>
       <c r="AO66" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP66" s="1" t="b">
         <v>1</v>
@@ -14714,7 +14711,7 @@
         <v>11</v>
       </c>
       <c r="AO67" s="1" t="s">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="AP67" s="1" t="b">
         <v>1</v>
@@ -14737,13 +14734,13 @@
         <v>600</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="H68" s="1">
         <v>1</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J68" s="1" t="s">
         <v>601</v>
@@ -14790,7 +14787,7 @@
         <v>4</v>
       </c>
       <c r="AO68" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP68" s="1" t="b">
         <v>1</v>
@@ -14819,7 +14816,7 @@
         <v>-1</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="J69" s="1" t="s">
         <v>606</v>
@@ -14863,7 +14860,7 @@
         <v>7</v>
       </c>
       <c r="AO69" s="1" t="s">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="AP69" s="1" t="b">
         <v>1</v>
@@ -15150,33 +15147,33 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>842</v>
+      </c>
+      <c r="B10" t="s">
         <v>843</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>844</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>845</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>846</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>847</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>848</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>849</v>
-      </c>
-      <c r="H10" t="s">
-        <v>850</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="B11" t="b">
         <v>1</v>
@@ -16193,6 +16190,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d56b9130-d22a-480d-bb83-f34040f04d96">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notes xmlns="d56b9130-d22a-480d-bb83-f34040f04d96" xsi:nil="true"/>
+    <TaxCatchAll xmlns="dd8606a3-d959-45f7-996e-3c98d970357c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010026B67AE13FBD584ABEFCF026840CED6F" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="11ebdf7d5c906124ef40ef85c2b08d8b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d56b9130-d22a-480d-bb83-f34040f04d96" xmlns:ns3="dd8606a3-d959-45f7-996e-3c98d970357c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="395e369db30c2620103728840cc29626" ns2:_="" ns3:_="">
     <xsd:import namespace="d56b9130-d22a-480d-bb83-f34040f04d96"/>
@@ -16461,42 +16479,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d56b9130-d22a-480d-bb83-f34040f04d96">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Notes xmlns="d56b9130-d22a-480d-bb83-f34040f04d96" xsi:nil="true"/>
-    <TaxCatchAll xmlns="dd8606a3-d959-45f7-996e-3c98d970357c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E038410E-E6A9-42FC-B223-5F20C9C2E8EB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D4B7956-BCA0-46CA-BF6B-C7215DA15D81}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="d56b9130-d22a-480d-bb83-f34040f04d96"/>
-    <ds:schemaRef ds:uri="dd8606a3-d959-45f7-996e-3c98d970357c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -16519,9 +16505,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D4B7956-BCA0-46CA-BF6B-C7215DA15D81}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E038410E-E6A9-42FC-B223-5F20C9C2E8EB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d56b9130-d22a-480d-bb83-f34040f04d96"/>
+    <ds:schemaRef ds:uri="dd8606a3-d959-45f7-996e-3c98d970357c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>